<commit_message>
improving the visibility of results
</commit_message>
<xml_diff>
--- a/resultados/posthoc_analysis.xlsx
+++ b/resultados/posthoc_analysis.xlsx
@@ -484,29 +484,45 @@
           <t>-</t>
         </is>
       </c>
-      <c r="C2" t="n">
-        <v>7.71164900840877e-07</v>
-      </c>
-      <c r="D2" t="n">
-        <v>2.802658150551885e-134</v>
-      </c>
-      <c r="E2" t="n">
-        <v>2.841648374042858e-05</v>
-      </c>
-      <c r="F2" t="n">
-        <v>0.01515105483989948</v>
-      </c>
-      <c r="G2" t="n">
-        <v>2.324650497121524e-31</v>
-      </c>
-      <c r="H2" t="n">
-        <v>0.001121309950490854</v>
-      </c>
-      <c r="I2" t="n">
-        <v>8.55648830017829e-07</v>
-      </c>
-      <c r="J2" t="n">
-        <v>7.065493628481349e-28</v>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>7.71e-07 ^</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2.8e-134 &lt;</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2.84e-05 ^</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>0.0152 &lt;</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>2.32e-31 &lt;</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>0.00112 &lt;</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>8.56e-07 ^</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>7.07e-28 &lt;</t>
+        </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -527,7 +543,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>7.71e-07 &lt;</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -535,36 +551,50 @@
           <t>-</t>
         </is>
       </c>
-      <c r="D3" t="n">
-        <v>1.272646012971163e-168</v>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>1.27e-168 &lt;</t>
+        </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F3" t="n">
-        <v>1.679662067603658e-11</v>
-      </c>
-      <c r="G3" t="n">
-        <v>6.548731490203138e-53</v>
-      </c>
-      <c r="H3" t="n">
-        <v>2.669409331755088e-14</v>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>1.68e-11 &lt;</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>6.55e-53 &lt;</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>2.67e-14 &lt;</t>
+        </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="J3" t="n">
-        <v>5.151620230867244e-48</v>
-      </c>
-      <c r="K3" t="n">
-        <v>2.198425186217402e-06</v>
-      </c>
-      <c r="L3" t="n">
-        <v>2.868749168840269e-06</v>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>5.15e-48 &lt;</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>2.2e-06 &lt;</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>2.87e-06 &lt;</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -575,12 +605,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2.8e-134 ^</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1.27e-168 ^</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -588,29 +618,45 @@
           <t>-</t>
         </is>
       </c>
-      <c r="E4" t="n">
-        <v>4.305242697150445e-165</v>
-      </c>
-      <c r="F4" t="n">
-        <v>5.898780855267603e-107</v>
-      </c>
-      <c r="G4" t="n">
-        <v>1.262864819735095e-49</v>
-      </c>
-      <c r="H4" t="n">
-        <v>4.722674358498086e-102</v>
-      </c>
-      <c r="I4" t="n">
-        <v>8.626372776065448e-165</v>
-      </c>
-      <c r="J4" t="n">
-        <v>1.554993741754963e-52</v>
-      </c>
-      <c r="K4" t="n">
-        <v>1.258896785018806e-121</v>
-      </c>
-      <c r="L4" t="n">
-        <v>2.568285894556331e-124</v>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>4.31e-165 ^</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>5.9e-107 ^</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>1.26e-49 ^</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>4.72e-102 ^</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>8.63e-165 ^</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>1.55e-52 ^</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>1.26e-121 ^</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2.57e-124 ^</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -621,7 +667,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2.84e-05 &lt;</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -631,7 +677,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>4.31e-165 &lt;</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -639,28 +685,40 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F5" t="n">
-        <v>1.415842429510318e-09</v>
-      </c>
-      <c r="G5" t="n">
-        <v>6.183425311217914e-50</v>
-      </c>
-      <c r="H5" t="n">
-        <v>1.676185714724637e-11</v>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>1.42e-09 &lt;</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>6.18e-50 &lt;</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>1.68e-11 &lt;</t>
+        </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="J5" t="n">
-        <v>1.201200527013148e-45</v>
-      </c>
-      <c r="K5" t="n">
-        <v>4.917063578377168e-05</v>
-      </c>
-      <c r="L5" t="n">
-        <v>0.0001069889847248471</v>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>1.2e-45 &lt;</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>4.92e-05 &lt;</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>0.000107 &lt;</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -671,22 +729,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0.0152 ^</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1.68e-11 ^</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>5.9e-107 &lt;</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1.42e-09 ^</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -694,25 +752,35 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G6" t="n">
-        <v>6.146109313037973e-19</v>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>6.15e-19 &lt;</t>
+        </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I6" t="n">
-        <v>3.536984577917394e-12</v>
-      </c>
-      <c r="J6" t="n">
-        <v>7.937770953464497e-18</v>
-      </c>
-      <c r="K6" t="n">
-        <v>0.02791461028247142</v>
-      </c>
-      <c r="L6" t="n">
-        <v>0.0192800351510725</v>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>3.54e-12 ^</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>7.94e-18 &lt;</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>0.0279 ^</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>0.0193 ^</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -723,27 +791,27 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2.32e-31 ^</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>6.55e-53 ^</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1.26e-49 &lt;</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>6.18e-50 ^</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>6.15e-19 ^</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -751,22 +819,30 @@
           <t>-</t>
         </is>
       </c>
-      <c r="H7" t="n">
-        <v>7.370807243538805e-17</v>
-      </c>
-      <c r="I7" t="n">
-        <v>7.090096206039435e-54</v>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>7.37e-17 ^</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>7.09e-54 ^</t>
+        </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K7" t="n">
-        <v>2.248077826259711e-28</v>
-      </c>
-      <c r="L7" t="n">
-        <v>1.035681077676983e-29</v>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>2.25e-28 ^</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>1.04e-29 ^</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -777,22 +853,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0.00112 ^</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2.67e-14 ^</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>4.72e-102 &lt;</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1.68e-11 ^</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -802,7 +878,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>7.37e-17 &lt;</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -810,17 +886,25 @@
           <t>-</t>
         </is>
       </c>
-      <c r="I8" t="n">
-        <v>1.228743420668558e-15</v>
-      </c>
-      <c r="J8" t="n">
-        <v>2.15906160208917e-14</v>
-      </c>
-      <c r="K8" t="n">
-        <v>0.005340992525067201</v>
-      </c>
-      <c r="L8" t="n">
-        <v>0.002130973557442648</v>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>1.23e-15 ^</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>2.16e-14 &lt;</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>0.00534 ^</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>0.00213 ^</t>
+        </is>
       </c>
     </row>
     <row r="9">
@@ -831,7 +915,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>8.56e-07 &lt;</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -841,7 +925,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>8.63e-165 &lt;</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -851,17 +935,17 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>3.54e-12 &lt;</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>7.09e-54 &lt;</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1.23e-15 &lt;</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -869,14 +953,20 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J9" t="n">
-        <v>9.00260127869011e-51</v>
-      </c>
-      <c r="K9" t="n">
-        <v>1.17056806136325e-06</v>
-      </c>
-      <c r="L9" t="n">
-        <v>1.811921749034463e-06</v>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>9e-51 &lt;</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>1.17e-06 &lt;</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>1.81e-06 &lt;</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -887,27 +977,27 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>7.07e-28 ^</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>5.15e-48 ^</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1.55e-52 &lt;</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1.2e-45 ^</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>7.94e-18 ^</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -917,12 +1007,12 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2.16e-14 ^</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>9e-51 ^</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -930,11 +1020,15 @@
           <t>-</t>
         </is>
       </c>
-      <c r="K10" t="n">
-        <v>4.835549187079496e-28</v>
-      </c>
-      <c r="L10" t="n">
-        <v>1.162198301147014e-27</v>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>4.84e-28 ^</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>1.16e-27 ^</t>
+        </is>
       </c>
     </row>
     <row r="11">
@@ -950,42 +1044,42 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2.2e-06 ^</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1.26e-121 &lt;</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>4.92e-05 ^</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0.0279 &lt;</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2.25e-28 &lt;</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0.00534 &lt;</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1.17e-06 ^</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>4.84e-28 &lt;</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1012,42 +1106,42 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2.87e-06 ^</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2.57e-124 &lt;</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0.000107 ^</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0.0193 &lt;</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1.04e-29 &lt;</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0.00213 &lt;</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1.81e-06 ^</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1.16e-27 &lt;</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">

</xml_diff>